<commit_message>
Pruebas y arreglos al codigo
</commit_message>
<xml_diff>
--- a/almacen_hospital.xlsx
+++ b/almacen_hospital.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,7 +462,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E2" t="n">
         <v>30</v>
@@ -508,6 +508,48 @@
       </c>
       <c r="E4" t="n">
         <v>30</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>108</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Omeprasol</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Medicamentos</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>60</v>
+      </c>
+      <c r="E5" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>187</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Doloneurobion</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Medicamentos</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>100</v>
+      </c>
+      <c r="E6" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -521,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -700,6 +742,78 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>101</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Reabastecimiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>101</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Salida</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Venta de medicamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>108</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Salida</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>40</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Venta de medicamento</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>